<commit_message>
Change LDO, Variant SMD_Assembly
</commit_message>
<xml_diff>
--- a/Project Outputs for Analog_MAX11331_Adapter_1v02/BOM/BOM_UltraZohm_Analog_Adapter_MAX11331_2v01.xlsx
+++ b/Project Outputs for Analog_MAX11331_Adapter_1v02/BOM/BOM_UltraZohm_Analog_Adapter_MAX11331_2v01.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hm-kreppel\Documents\Altium Projects\ultrazohm_analog_max11331_main_1vxx\Project Outputs for Analog_MAX11331_Adapter_1v02\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\Documents\Altium\UltraZOhm\UZ_A_MAX1131_Adapter\Project Outputs for Analog_MAX11331_Adapter_1v02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F870D097-9E90-4CC9-A0E2-E66554A83297}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="11565"/>
+    <workbookView xWindow="1500" yWindow="180" windowWidth="21600" windowHeight="11385" xr2:uid="{87A741BB-0D20-4D2E-A066-7576B3F453B1}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UltraZohm_Analog_Adapter_MA" sheetId="1" r:id="rId1"/>
@@ -17,17 +18,26 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">BOM_UltraZohm_Analog_Adapter_MA!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="158">
   <si>
     <t>Name</t>
   </si>
@@ -173,27 +183,6 @@
     <t>C0603C122K5RACTU</t>
   </si>
   <si>
-    <t>68µF</t>
-  </si>
-  <si>
-    <t>C8, C9</t>
-  </si>
-  <si>
-    <t>WCAP-ATG8 THT Aluminum Electrolytic Capacitors, D6.3mm x L11mm, 68uF, +/-20%, 35VDC</t>
-  </si>
-  <si>
-    <t>+/-20%</t>
-  </si>
-  <si>
-    <t>WCAP-ATG8_6.3x11</t>
-  </si>
-  <si>
-    <t>732-8736-1-ND</t>
-  </si>
-  <si>
-    <t>860010573006</t>
-  </si>
-  <si>
     <t>10µF</t>
   </si>
   <si>
@@ -266,7 +255,7 @@
     <t>WL-SMCW SMT Mono-color Chip LED Waterclear, size 0603, Blue, 3.2V, 140deg</t>
   </si>
   <si>
-    <t>732-4966-1-ND</t>
+    <t>732-4966-6-ND</t>
   </si>
   <si>
     <t>150060BS75000</t>
@@ -398,7 +387,7 @@
     <t>R29</t>
   </si>
   <si>
-    <t>311-100KHRCT-ND</t>
+    <t>311-100KHRDKR-ND</t>
   </si>
   <si>
     <t>RC0603FR-07100KL</t>
@@ -440,121 +429,94 @@
     <t>TSOP65P640X120-16N</t>
   </si>
   <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>296-24739-1-ND</t>
+    <t>296-23611-5-ND</t>
+  </si>
+  <si>
+    <t>Rochester Electronics</t>
+  </si>
+  <si>
+    <t>SN74AVC4T774PW</t>
+  </si>
+  <si>
+    <t>Quad LVDS driver</t>
+  </si>
+  <si>
+    <t>U2A, U2B, U2C</t>
+  </si>
+  <si>
+    <t>3V, LVDS, Quad, CMOS Differential Line Driver</t>
+  </si>
+  <si>
+    <t>ADN4665ARUZ-ND</t>
+  </si>
+  <si>
+    <t>Analog Devices</t>
+  </si>
+  <si>
+    <t>ADN4665ARUZ</t>
+  </si>
+  <si>
+    <t>Quad LVDS reciever</t>
+  </si>
+  <si>
+    <t>U3A, U3B, U3C</t>
+  </si>
+  <si>
+    <t>3V, LVDS, quad, CMOS Differential Line Receiver</t>
+  </si>
+  <si>
+    <t>ADN4666ARUZ-ND</t>
+  </si>
+  <si>
+    <t>ADN4666ARUZ</t>
+  </si>
+  <si>
+    <t>buck converter</t>
+  </si>
+  <si>
+    <t>U5</t>
+  </si>
+  <si>
+    <t>100V Input, 0.5A Synchronous Buck DC/DC Converter with Ultra-low Iq</t>
+  </si>
+  <si>
+    <t>SOIC127P600X170_HS-9N</t>
+  </si>
+  <si>
+    <t>296-LM5163HQDDARQ1CT-ND</t>
   </si>
   <si>
     <t>Texas Instruments</t>
   </si>
   <si>
-    <t>SN74AVC4T774PWR</t>
-  </si>
-  <si>
-    <t>Quad LVDS driver</t>
-  </si>
-  <si>
-    <t>U2A, U2B, U2C</t>
-  </si>
-  <si>
-    <t>3V, LVDS, Quad, CMOS Differential Line Driver</t>
-  </si>
-  <si>
-    <t>ADN4665ARUZ-ND</t>
-  </si>
-  <si>
-    <t>Analog Devices</t>
-  </si>
-  <si>
-    <t>ADN4665ARUZ</t>
-  </si>
-  <si>
-    <t>Quad LVDS reciever</t>
-  </si>
-  <si>
-    <t>U3A, U3B, U3C</t>
-  </si>
-  <si>
-    <t>3V, LVDS, quad, CMOS Differential Line Receiver</t>
-  </si>
-  <si>
-    <t>ADN4666ARUZ-ND</t>
-  </si>
-  <si>
-    <t>ADN4666ARUZ</t>
-  </si>
-  <si>
-    <t>buck converter</t>
-  </si>
-  <si>
-    <t>U5</t>
-  </si>
-  <si>
-    <t>100V Input, 0.5A Synchronous Buck DC/DC Converter with Ultra-low Iq</t>
-  </si>
-  <si>
-    <t>SOIC127P600X170_HS-9N</t>
-  </si>
-  <si>
-    <t>296-LM5163HQDDARQ1CT-ND</t>
-  </si>
-  <si>
     <t>LM5163HQDDARQ1</t>
   </si>
   <si>
-    <t>LDO</t>
+    <t>1.8V LDO</t>
   </si>
   <si>
     <t>U6</t>
   </si>
   <si>
-    <t>0.3A Low-Dropout Regulator</t>
-  </si>
-  <si>
-    <t>SOT-23-5</t>
-  </si>
-  <si>
-    <t>296-48712-1-ND</t>
-  </si>
-  <si>
-    <t>TLV74318PDBVR</t>
-  </si>
-  <si>
-    <t>2x8 Pin</t>
-  </si>
-  <si>
-    <t>X2A, X2B, X2C</t>
-  </si>
-  <si>
-    <t>Dual Row, 2x8 Shrouded IDC Header with Ejectors 50 mil pitch</t>
-  </si>
-  <si>
-    <t>EHF-108-01-F-D</t>
-  </si>
-  <si>
-    <t>SAM9265-ND</t>
-  </si>
-  <si>
-    <t>Samtec</t>
-  </si>
-  <si>
-    <t>IPL1-102-01-L-D-K</t>
-  </si>
-  <si>
-    <t>X3, X4, X5</t>
-  </si>
-  <si>
-    <t>2.54mm Double Row Terminal Assembly, Right-Angled</t>
-  </si>
-  <si>
-    <t>SAM10565-ND</t>
+    <t>1A Positive 1.8V Fixed-Voltage Low-Dropout Regulator</t>
+  </si>
+  <si>
+    <t>SOT230P700X170-4N</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>595-TLV1117-15IDCYR</t>
+  </si>
+  <si>
+    <t>TLV1117-15IDCYR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -651,7 +613,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -663,7 +625,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -710,6 +672,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -745,6 +724,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -896,11 +892,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ACE7A68-7062-42B2-9862-C833CEC83236}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
@@ -1158,7 +1154,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="135" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -1169,100 +1165,104 @@
         <v>48</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="3" t="s">
+      <c r="H6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H6" s="4"/>
-      <c r="I6" s="3" t="s">
+      <c r="L6" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K6" s="3" t="s">
+      <c r="M6" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="L6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M6" s="3" t="s">
-        <v>54</v>
-      </c>
       <c r="N6" s="4">
-        <v>0.13</v>
+        <v>0.32</v>
       </c>
       <c r="O6" s="4">
         <v>2</v>
       </c>
       <c r="P6" s="4">
-        <v>0.26</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="C7" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>31</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M7" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="L7" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="N7" s="4">
-        <v>0.32</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="O7" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P7" s="4">
-        <v>0.64</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>38</v>
@@ -1271,13 +1271,13 @@
         <v>28</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>32</v>
@@ -1286,84 +1286,76 @@
         <v>21</v>
       </c>
       <c r="K8" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="N8" s="4">
+        <v>0.12</v>
+      </c>
+      <c r="O8" s="4">
+        <v>1</v>
+      </c>
+      <c r="P8" s="4">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="L8" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M8" s="3" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="N8" s="4">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="O8" s="4">
-        <v>3</v>
-      </c>
-      <c r="P8" s="4">
-        <v>0.84</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>38</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>45</v>
-      </c>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
       <c r="I9" s="3" t="s">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K9" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M9" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="L9" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>69</v>
-      </c>
       <c r="N9" s="4">
-        <v>0.12</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O9" s="4">
         <v>1</v>
       </c>
       <c r="P9" s="4">
-        <v>0.12</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>28</v>
@@ -1372,40 +1364,40 @@
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="3" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="N10" s="4">
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="O10" s="4">
         <v>1</v>
       </c>
       <c r="P10" s="4">
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>28</v>
@@ -1414,73 +1406,73 @@
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="3" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="N11" s="4">
-        <v>0.16</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O11" s="4">
         <v>1</v>
       </c>
       <c r="P11" s="4">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>28</v>
-      </c>
+      <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="3" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K12" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="L12" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>85</v>
       </c>
       <c r="N12" s="4">
-        <v>0.14000000000000001</v>
+        <v>0.33</v>
       </c>
       <c r="O12" s="4">
         <v>1</v>
       </c>
       <c r="P12" s="4">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -1493,208 +1485,212 @@
       <c r="D13" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
+      <c r="E13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="N13" s="4">
-        <v>0.33</v>
+        <v>0.1</v>
       </c>
       <c r="O13" s="4">
         <v>1</v>
       </c>
       <c r="P13" s="4">
-        <v>0.33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="D14" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="M14" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="J14" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K14" s="3" t="s">
+      <c r="N14" s="4">
+        <v>2.4E-2</v>
+      </c>
+      <c r="O14" s="4">
+        <v>21</v>
+      </c>
+      <c r="P14" s="4">
+        <v>0.504</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="L14" s="3" t="s">
+      <c r="B15" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="M14" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="N14" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="O14" s="4">
-        <v>1</v>
-      </c>
-      <c r="P14" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>102</v>
-      </c>
       <c r="C15" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="N15" s="4">
         <v>2.4E-2</v>
       </c>
       <c r="O15" s="4">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="P15" s="4">
-        <v>0.504</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>0.38400000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="N16" s="4">
-        <v>2.4E-2</v>
+        <v>0.1</v>
       </c>
       <c r="O16" s="4">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="P16" s="4">
-        <v>0.38400000000000001</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="N17" s="4">
         <v>0.1</v>
@@ -1708,39 +1704,39 @@
     </row>
     <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="N18" s="4">
         <v>0.1</v>
@@ -1754,39 +1750,39 @@
     </row>
     <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="N19" s="4">
         <v>0.1</v>
@@ -1800,39 +1796,39 @@
     </row>
     <row r="20" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="N20" s="4">
         <v>0.1</v>
@@ -1846,39 +1842,39 @@
     </row>
     <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="N21" s="4">
         <v>0.1</v>
@@ -1890,53 +1886,47 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="210" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="C22" s="4"/>
       <c r="D22" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>96</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="3" t="s">
-        <v>97</v>
+        <v>129</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K22" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="L22" s="3" t="s">
         <v>131</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>99</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>132</v>
       </c>
       <c r="N22" s="4">
-        <v>0.1</v>
+        <v>1.39</v>
       </c>
       <c r="O22" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P22" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" ht="210" x14ac:dyDescent="0.25">
+        <v>6.95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>133</v>
       </c>
@@ -1952,55 +1942,59 @@
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K23" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="J23" s="3" t="s">
+      <c r="L23" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="K23" s="3" t="s">
+      <c r="M23" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="L23" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="M23" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="N23" s="4"/>
+      <c r="N23" s="4">
+        <v>3.34</v>
+      </c>
       <c r="O23" s="4">
-        <v>5</v>
-      </c>
-      <c r="P23" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="P23" s="4">
+        <v>10.02</v>
+      </c>
     </row>
     <row r="24" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="N24" s="4">
         <v>3.34</v>
@@ -2012,207 +2006,89 @@
         <v>10.02</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="105" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="3" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="3" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K25" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="M25" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="L25" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="M25" s="3" t="s">
+      <c r="N25" s="4">
+        <v>4.49</v>
+      </c>
+      <c r="O25" s="4">
+        <v>1</v>
+      </c>
+      <c r="P25" s="4">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="N25" s="4">
-        <v>3.34</v>
-      </c>
-      <c r="O25" s="4">
-        <v>3</v>
-      </c>
-      <c r="P25" s="4">
-        <v>10.02</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" ht="105" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>152</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>153</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
       <c r="I26" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="J26" s="3" t="s">
         <v>155</v>
-      </c>
-      <c r="J26" s="3" t="s">
-        <v>21</v>
       </c>
       <c r="K26" s="3" t="s">
         <v>156</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>157</v>
       </c>
       <c r="N26" s="4">
-        <v>4.49</v>
+        <v>0.71</v>
       </c>
       <c r="O26" s="4">
         <v>1</v>
       </c>
       <c r="P26" s="4">
-        <v>4.49</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="K27" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="L27" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="M27" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="N27" s="4"/>
-      <c r="O27" s="4">
-        <v>1</v>
-      </c>
-      <c r="P27" s="4"/>
-    </row>
-    <row r="28" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K28" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="L28" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="M28" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="N28" s="4">
-        <v>4.8499999999999996</v>
-      </c>
-      <c r="O28" s="4">
-        <v>3</v>
-      </c>
-      <c r="P28" s="4">
-        <v>14.55</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K29" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="L29" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="M29" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="N29" s="4">
-        <v>3.64</v>
-      </c>
-      <c r="O29" s="4">
-        <v>3</v>
-      </c>
-      <c r="P29" s="4">
-        <v>10.92</v>
+        <v>0.71</v>
       </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="30" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="35" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>